<commit_message>
Default to Thai, explain target home cards, update logic summary
Sets Thai as the app's default language, adds (i) tooltips explaining
the logic behind the 3 target-home cards, and shows the target home
price's loan + down payment breakdown. Also brings the Logic Summary
workbook up to date with the recently added Net Cash Flow calculation.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Home-Ready-Logic-Summary.xlsx
+++ b/Home-Ready-Logic-Summary.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A101"/>
+  <dimension ref="A1:A105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -892,7 +892,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">                                Remaining Monthly Income, cushion status, Initial Payment, Total Paid Over 10 Years).</t>
+          <t xml:space="preserve">                                Remaining Monthly Income, cushion status, Initial Payment, Total Paid Over 10 Years, Capital Value, and Net Cash Flow over 10 Years (calculateNetCashFlow10Years).</t>
         </is>
       </c>
     </row>
@@ -1330,23 +1330,51 @@
         </is>
       </c>
     </row>
-    <row r="98"/>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Added a Net Cash Flow over 10 Years row to the Cash Flow comparison (Sheet 9a/9b, row 13):</t>
+        </is>
+      </c>
+    </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Two reference spreadsheets already in this project informed parts of this logic and are worth cross-checking too:</t>
+          <t xml:space="preserve">    Capital Value minus Total Paid, sign-colored — the single bottom-line figure netting equity built</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • RTO-Payment.xlsx — the authoritative source for every Rent-to-Own formula (Sheets 8a/8b reproduce it exactly).</t>
+          <t xml:space="preserve">    against cash spent (calculateNetCashFlow10Years). Rent's Capital Value counts as ฿0 (it never</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    accumulates), so Rent's Net Cash Flow reduces to exactly negative Total Paid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102"/>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Two reference spreadsheets already in this project informed parts of this logic and are worth cross-checking too:</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • RTO-Payment.xlsx — the authoritative source for every Rent-to-Own formula (Sheets 8a/8b reproduce it exactly).</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
         <is>
           <t xml:space="preserve">  • Home-Ready-Calculation-Audit.xlsx — an earlier audit pass.</t>
         </is>
@@ -4092,7 +4120,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -4115,7 +4143,7 @@
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="33" t="inlineStr">
         <is>
-          <t>"Remaining Monthly Income" = Income After Other Obligations (Sheet 3) minus THIS option's own monthly housing payment — bonus excluded, debt/living-expenses/lump-sum already excluded upstream in Sheet 3. Row 11 (Total Paid Over 10 Years): Rent reads Sheet 7's own growing cumulative total (not a flat multiply — rent grows with property appreciation); RTO reads Sheet 8's Total Paid Over 10 Years (RTO), which itself splits into 3 years of RTO payments + 7 years of a post-transition mortgage — never a flat monthly payment for all 10 years. Buy alone stays a flat multiply (a mortgage installment genuinely is fixed for its whole term).</t>
+          <t>"Remaining Monthly Income" = Income After Other Obligations (Sheet 3) minus THIS option's own monthly housing payment — bonus excluded, debt/living-expenses/lump-sum already excluded upstream in Sheet 3. Row 11 (Total Paid Over 10 Years): Rent reads Sheet 7's own growing cumulative total (not a flat multiply — rent grows with property appreciation); RTO reads Sheet 8's Total Paid Over 10 Years (RTO), which itself splits into 3 years of RTO payments + 7 years of a post-transition mortgage — never a flat monthly payment for all 10 years. Buy alone stays a flat multiply (a mortgage installment genuinely is fixed for its whole term). Row 13 (Net Cash Flow over 10 Years) is Capital Value minus Total Paid (calculateNetCashFlow10Years) — Rent's Capital Value counts as ฿0 since it never accumulates, so Rent's Net Cash Flow is simply its Total Paid, negated.</t>
         </is>
       </c>
     </row>
@@ -4271,10 +4299,30 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Row references used elsewhere: Remaining Monthly Income row = 7, Cushion Status row = 9, Remaining % row = 8.</t>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Net Cash Flow over 10 Years</t>
+        </is>
+      </c>
+      <c r="B13" s="32">
+        <f>0-B11</f>
+        <v/>
+      </c>
+      <c r="C13" s="32">
+        <f>C12-C11</f>
+        <v/>
+      </c>
+      <c r="D13" s="32">
+        <f>D12-D11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1"/>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Row references used elsewhere: Remaining Monthly Income row = 7, Cushion Status row = 9, Remaining % row = 8, Net Cash Flow row = 13.</t>
         </is>
       </c>
     </row>
@@ -4294,7 +4342,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -4317,7 +4365,7 @@
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="33" t="inlineStr">
         <is>
-          <t>"Remaining Monthly Income" = Income After Other Obligations (Sheet 3) minus THIS option's own monthly housing payment — bonus excluded, debt/living-expenses/lump-sum already excluded upstream in Sheet 3. Row 11 (Total Paid Over 10 Years): Rent reads Sheet 7's own growing cumulative total (not a flat multiply — rent grows with property appreciation); RTO reads Sheet 8's Total Paid Over 10 Years (RTO), which itself splits into 3 years of RTO payments + 7 years of a post-transition mortgage — never a flat monthly payment for all 10 years. Buy alone stays a flat multiply (a mortgage installment genuinely is fixed for its whole term).</t>
+          <t>"Remaining Monthly Income" = Income After Other Obligations (Sheet 3) minus THIS option's own monthly housing payment — bonus excluded, debt/living-expenses/lump-sum already excluded upstream in Sheet 3. Row 11 (Total Paid Over 10 Years): Rent reads Sheet 7's own growing cumulative total (not a flat multiply — rent grows with property appreciation); RTO reads Sheet 8's Total Paid Over 10 Years (RTO), which itself splits into 3 years of RTO payments + 7 years of a post-transition mortgage — never a flat monthly payment for all 10 years. Buy alone stays a flat multiply (a mortgage installment genuinely is fixed for its whole term). Row 13 (Net Cash Flow over 10 Years) is Capital Value minus Total Paid (calculateNetCashFlow10Years) — Rent's Capital Value counts as ฿0 since it never accumulates, so Rent's Net Cash Flow is simply its Total Paid, negated.</t>
         </is>
       </c>
     </row>
@@ -4473,10 +4521,30 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Row references used elsewhere: Remaining Monthly Income row = 7, Cushion Status row = 9, Remaining % row = 8.</t>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Net Cash Flow over 10 Years</t>
+        </is>
+      </c>
+      <c r="B13" s="32">
+        <f>0-B11</f>
+        <v/>
+      </c>
+      <c r="C13" s="32">
+        <f>C12-C11</f>
+        <v/>
+      </c>
+      <c r="D13" s="32">
+        <f>D12-D11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1"/>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Row references used elsewhere: Remaining Monthly Income row = 7, Cushion Status row = 9, Remaining % row = 8, Net Cash Flow row = 13.</t>
         </is>
       </c>
     </row>

</xml_diff>